<commit_message>
Se ingresa nuevo participante
</commit_message>
<xml_diff>
--- a/mundial_2026_apuestas.xlsx
+++ b/mundial_2026_apuestas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1fe95bc314a61fb9/Jupyter/Proyectos/Resultados Mundial 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{355737B5-6343-4C2A-84AC-C8F379D8C966}"/>
+  <xr:revisionPtr revIDLastSave="99" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96605314-B40E-45D9-B053-0D59D2B7C5D3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="66">
   <si>
     <t>⚽  MUNDIAL 2026 — CONTROL DE APUESTAS</t>
   </si>
@@ -234,6 +234,9 @@
   </si>
   <si>
     <t>Efectivo</t>
+  </si>
+  <si>
+    <t>Por Definir</t>
   </si>
 </sst>
 </file>
@@ -505,20 +508,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -661,6 +652,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -746,6 +752,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -939,402 +949,414 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
+      <c r="A1" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="49"/>
     </row>
     <row r="2" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
     </row>
     <row r="3" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="15" t="s">
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="51"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="16" t="s">
+      <c r="G4" s="47"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="12" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="52">
+      <c r="G5" s="48">
         <v>46175</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="H5" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="I5" s="13"/>
+      <c r="I5" s="9"/>
     </row>
     <row r="6" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="51">
+      <c r="G6" s="47">
         <v>46174</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="I6" s="10"/>
+      <c r="I6" s="6"/>
     </row>
     <row r="7" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="52">
+      <c r="G7" s="48">
         <v>46174</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="I7" s="13"/>
+      <c r="I7" s="9"/>
     </row>
     <row r="8" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="51">
+      <c r="G8" s="47">
         <v>46176</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="I8" s="10"/>
+      <c r="I8" s="6"/>
     </row>
     <row r="9" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="52">
+      <c r="G9" s="48">
         <v>46175</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="I9" s="13"/>
+      <c r="I9" s="9"/>
     </row>
     <row r="10" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="15" t="s">
+      <c r="B10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="47">
+        <v>46178</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="I10" s="6"/>
+    </row>
+    <row r="11" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="48">
+        <v>46174</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" s="9"/>
+    </row>
+    <row r="12" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="47">
+        <v>46176</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="I12" s="6"/>
+    </row>
+    <row r="13" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="51"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="16" t="s">
+      <c r="G13" s="48"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" s="14" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="47">
+        <v>46175</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="I14" s="6"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="48"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="F11" s="12" t="s">
+      <c r="C16" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="52">
-        <v>46174</v>
-      </c>
-      <c r="H11" s="14" t="s">
+      <c r="G16" s="47">
+        <v>46176</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="I16" s="6"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G17" s="48">
+        <v>46178</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="I11" s="13"/>
-    </row>
-    <row r="12" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" s="51">
-        <v>46176</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="I12" s="10"/>
-    </row>
-    <row r="13" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="15" t="s">
+      <c r="I17" s="9"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="52"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="G14" s="51">
-        <v>46175</v>
-      </c>
-      <c r="H14" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="I14" s="10"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G15" s="52"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="G16" s="51">
-        <v>46176</v>
-      </c>
-      <c r="H16" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="I16" s="10"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G17" s="52"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G18" s="51"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="16" t="s">
+      <c r="G18" s="47"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="12" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1359,63 +1381,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
     </row>
     <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
     </row>
     <row r="3" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="13" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="20">
+      <c r="B4" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="16">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="20">
+      <c r="B5" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="16">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="20">
+      <c r="B6" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="16">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="20">
+      <c r="B7" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="16">
         <v>1</v>
       </c>
     </row>
@@ -1441,354 +1471,354 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
     </row>
     <row r="3" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="24">
+      <c r="A4" s="20">
         <v>1</v>
       </c>
-      <c r="B4" s="25" t="str">
+      <c r="B4" s="21" t="str">
         <f>Apuestas!A4</f>
         <v>Carlos</v>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="22">
         <f>IF(Apuestas!B4='Resultados Oficiales'!$B$4,4,0)</f>
-        <v>4</v>
-      </c>
-      <c r="D4" s="26">
+        <v>0</v>
+      </c>
+      <c r="D4" s="22">
         <f>IF(Apuestas!C4='Resultados Oficiales'!$B$5,3,0)</f>
-        <v>3</v>
-      </c>
-      <c r="E4" s="26">
+        <v>0</v>
+      </c>
+      <c r="E4" s="22">
         <f>IF(Apuestas!D4='Resultados Oficiales'!$B$6,2,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="22">
+        <f>IF(Apuestas!E4='Resultados Oficiales'!$B$7,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="23">
+        <f t="shared" ref="G4:G13" si="0">SUM(C4:F4)</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="22"/>
+    </row>
+    <row r="5" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="24">
         <v>2</v>
       </c>
-      <c r="F4" s="26">
-        <f>IF(Apuestas!E4='Resultados Oficiales'!$B$7,1,0)</f>
-        <v>1</v>
-      </c>
-      <c r="G4" s="27">
-        <f t="shared" ref="G4:G13" si="0">SUM(C4:F4)</f>
-        <v>10</v>
-      </c>
-      <c r="H4" s="26"/>
-    </row>
-    <row r="5" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="28">
-        <v>2</v>
-      </c>
-      <c r="B5" s="29" t="str">
+      <c r="B5" s="25" t="str">
         <f>Apuestas!A5</f>
         <v>Cristian</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="26">
         <f>IF(Apuestas!B5='Resultados Oficiales'!$B$4,4,0)</f>
         <v>0</v>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="26">
         <f>IF(Apuestas!C5='Resultados Oficiales'!$B$5,3,0)</f>
         <v>0</v>
       </c>
-      <c r="E5" s="30">
+      <c r="E5" s="26">
         <f>IF(Apuestas!D5='Resultados Oficiales'!$B$6,2,0)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="30">
+      <c r="F5" s="26">
         <f>IF(Apuestas!E5='Resultados Oficiales'!$B$7,1,0)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="31">
+      <c r="G5" s="27">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H5" s="30"/>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="32">
+      <c r="A6" s="28">
         <v>3</v>
       </c>
-      <c r="B6" s="33" t="str">
+      <c r="B6" s="29" t="str">
         <f>Apuestas!A6</f>
         <v>Cristian Jr.</v>
       </c>
-      <c r="C6" s="34">
+      <c r="C6" s="30">
         <f>IF(Apuestas!B6='Resultados Oficiales'!$B$4,4,0)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="34">
+      <c r="D6" s="30">
         <f>IF(Apuestas!C6='Resultados Oficiales'!$B$5,3,0)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="34">
+      <c r="E6" s="30">
         <f>IF(Apuestas!D6='Resultados Oficiales'!$B$6,2,0)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="34">
+      <c r="F6" s="30">
         <f>IF(Apuestas!E6='Resultados Oficiales'!$B$7,1,0)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="35">
+      <c r="G6" s="31">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="34"/>
+      <c r="H6" s="30"/>
     </row>
     <row r="7" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="36">
+      <c r="A7" s="32">
         <v>4</v>
       </c>
-      <c r="B7" s="37" t="str">
+      <c r="B7" s="33" t="str">
         <f>Apuestas!A7</f>
         <v>Dany</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="7">
         <f>IF(Apuestas!B7='Resultados Oficiales'!$B$4,4,0)</f>
         <v>0</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="7">
         <f>IF(Apuestas!C7='Resultados Oficiales'!$B$5,3,0)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="7">
         <f>IF(Apuestas!D7='Resultados Oficiales'!$B$6,2,0)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="7">
         <f>IF(Apuestas!E7='Resultados Oficiales'!$B$7,1,0)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="38">
+      <c r="G7" s="34">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="39">
+      <c r="A8" s="35">
         <v>5</v>
       </c>
-      <c r="B8" s="40" t="str">
+      <c r="B8" s="36" t="str">
         <f>Apuestas!A8</f>
         <v>Dino</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="10">
         <f>IF(Apuestas!B8='Resultados Oficiales'!$B$4,4,0)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="10">
         <f>IF(Apuestas!C8='Resultados Oficiales'!$B$5,3,0)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="10">
         <f>IF(Apuestas!D8='Resultados Oficiales'!$B$6,2,0)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="10">
         <f>IF(Apuestas!E8='Resultados Oficiales'!$B$7,1,0)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="41">
+      <c r="G8" s="37">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="14"/>
+      <c r="H8" s="10"/>
     </row>
     <row r="9" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="36">
+      <c r="A9" s="32">
         <v>6</v>
       </c>
-      <c r="B9" s="37" t="str">
+      <c r="B9" s="33" t="str">
         <f>Apuestas!A9</f>
         <v>Don Segundo</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="7">
         <f>IF(Apuestas!B9='Resultados Oficiales'!$B$4,4,0)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="7">
         <f>IF(Apuestas!C9='Resultados Oficiales'!$B$5,3,0)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="7">
         <f>IF(Apuestas!D9='Resultados Oficiales'!$B$6,2,0)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="7">
         <f>IF(Apuestas!E9='Resultados Oficiales'!$B$7,1,0)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="38">
+      <c r="G9" s="34">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="39">
+      <c r="A10" s="35">
         <v>7</v>
       </c>
-      <c r="B10" s="40" t="str">
+      <c r="B10" s="36" t="str">
         <f>Apuestas!A10</f>
         <v>Fabian</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="10">
         <f>IF(Apuestas!B10='Resultados Oficiales'!$B$4,4,0)</f>
-        <v>4</v>
-      </c>
-      <c r="D10" s="14">
+        <v>0</v>
+      </c>
+      <c r="D10" s="10">
         <f>IF(Apuestas!C10='Resultados Oficiales'!$B$5,3,0)</f>
-        <v>3</v>
-      </c>
-      <c r="E10" s="14">
+        <v>0</v>
+      </c>
+      <c r="E10" s="10">
         <f>IF(Apuestas!D10='Resultados Oficiales'!$B$6,2,0)</f>
-        <v>2</v>
-      </c>
-      <c r="F10" s="14">
+        <v>0</v>
+      </c>
+      <c r="F10" s="10">
         <f>IF(Apuestas!E10='Resultados Oficiales'!$B$7,1,0)</f>
-        <v>1</v>
-      </c>
-      <c r="G10" s="41">
+        <v>0</v>
+      </c>
+      <c r="G10" s="37">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="H10" s="14"/>
+        <v>0</v>
+      </c>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="36">
+      <c r="A11" s="32">
         <v>8</v>
       </c>
-      <c r="B11" s="37" t="str">
+      <c r="B11" s="33" t="str">
         <f>Apuestas!A11</f>
         <v>JM</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="7">
         <f>IF(Apuestas!B11='Resultados Oficiales'!$B$4,4,0)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="7">
         <f>IF(Apuestas!C11='Resultados Oficiales'!$B$5,3,0)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="7">
         <f>IF(Apuestas!D11='Resultados Oficiales'!$B$6,2,0)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="11">
+      <c r="F11" s="7">
         <f>IF(Apuestas!E11='Resultados Oficiales'!$B$7,1,0)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="38">
+      <c r="G11" s="34">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H11" s="11"/>
+      <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="39">
+      <c r="A12" s="35">
         <v>9</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="36" t="str">
         <f>Apuestas!A12</f>
         <v>Juan Reveco</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="10">
         <f>IF(Apuestas!B12='Resultados Oficiales'!$B$4,4,0)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="10">
         <f>IF(Apuestas!C12='Resultados Oficiales'!$B$5,3,0)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="10">
         <f>IF(Apuestas!D12='Resultados Oficiales'!$B$6,2,0)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="14">
+      <c r="F12" s="10">
         <f>IF(Apuestas!E12='Resultados Oficiales'!$B$7,1,0)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="41">
+      <c r="G12" s="37">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="14"/>
+      <c r="H12" s="10"/>
     </row>
     <row r="13" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="36">
+      <c r="A13" s="32">
         <v>10</v>
       </c>
-      <c r="B13" s="37" t="str">
+      <c r="B13" s="33" t="str">
         <f>Apuestas!A13</f>
         <v>Kote</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="7">
         <f>IF(Apuestas!B13='Resultados Oficiales'!$B$4,4,0)</f>
-        <v>4</v>
-      </c>
-      <c r="D13" s="11">
+        <v>0</v>
+      </c>
+      <c r="D13" s="7">
         <f>IF(Apuestas!C13='Resultados Oficiales'!$B$5,3,0)</f>
-        <v>3</v>
-      </c>
-      <c r="E13" s="11">
+        <v>0</v>
+      </c>
+      <c r="E13" s="7">
         <f>IF(Apuestas!D13='Resultados Oficiales'!$B$6,2,0)</f>
-        <v>2</v>
-      </c>
-      <c r="F13" s="11">
+        <v>0</v>
+      </c>
+      <c r="F13" s="7">
         <f>IF(Apuestas!E13='Resultados Oficiales'!$B$7,1,0)</f>
-        <v>1</v>
-      </c>
-      <c r="G13" s="38">
+        <v>0</v>
+      </c>
+      <c r="G13" s="34">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="H13" s="11"/>
+        <v>0</v>
+      </c>
+      <c r="H13" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1811,69 +1841,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
     </row>
     <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="43">
-        <f>COUNTIF(Apuestas!F4:F13,"✓ Sí")</f>
-        <v>7</v>
-      </c>
-      <c r="C2" s="44"/>
+      <c r="B2" s="53">
+        <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")</f>
+        <v>10</v>
+      </c>
+      <c r="C2" s="40"/>
     </row>
     <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="46">
-        <f>COUNTIF(Apuestas!F4:F13,"✓ Sí")*100000</f>
-        <v>700000</v>
-      </c>
-      <c r="C3" s="47"/>
+      <c r="B3" s="42">
+        <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")*100000</f>
+        <v>1000000</v>
+      </c>
+      <c r="C3" s="43"/>
     </row>
     <row r="4" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="48"/>
-      <c r="B4" s="49"/>
-      <c r="C4" s="44"/>
+      <c r="A4" s="44"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="40"/>
     </row>
     <row r="5" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="46">
-        <f>COUNTIF(Apuestas!F4:F13,"✓ Sí")*100000-100000</f>
-        <v>600000</v>
-      </c>
-      <c r="C5" s="50" t="s">
+      <c r="B5" s="42">
+        <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")*100000-100000</f>
+        <v>900000</v>
+      </c>
+      <c r="C5" s="46" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="42" t="s">
+      <c r="A6" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="43">
+      <c r="B6" s="39">
         <v>100000</v>
       </c>
-      <c r="C6" s="50" t="s">
+      <c r="C6" s="46" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="46">
+      <c r="B7" s="42">
         <f>B5+B6</f>
-        <v>700000</v>
-      </c>
-      <c r="C7" s="47"/>
+        <v>1000000</v>
+      </c>
+      <c r="C7" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Se actualiza apuesta incorrecta
</commit_message>
<xml_diff>
--- a/mundial_2026_apuestas.xlsx
+++ b/mundial_2026_apuestas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1fe95bc314a61fb9/Jupyter/Proyectos/Resultados Mundial 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="118" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAD711BE-237C-43E1-97FB-B9EE82DBA51F}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49CA2F73-0FBD-4D08-8051-AF12086D5F58}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1100,7 +1100,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>14</v>
@@ -1114,10 +1114,10 @@
       <c r="I6" s="6"/>
       <c r="J6" t="str">
         <f t="shared" si="0"/>
-        <v>Francia-España-Argentina-Inglaterra</v>
+        <v>Francia-España-Argentina-Portugal</v>
       </c>
       <c r="K6" t="str">
-        <v>Francia-España-Argentina-Inglaterra</v>
+        <v>Francia-España-Argentina-Portugal</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Se actualizan apuestas y apostadores
</commit_message>
<xml_diff>
--- a/mundial_2026_apuestas.xlsx
+++ b/mundial_2026_apuestas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1fe95bc314a61fb9/Jupyter/Proyectos/Resultados Mundial 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49CA2F73-0FBD-4D08-8051-AF12086D5F58}"/>
+  <xr:revisionPtr revIDLastSave="131" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0036DAEC-E792-4BFC-9289-A46DAFEAF869}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="66">
   <si>
     <t>⚽  MUNDIAL 2026 — CONTROL DE APUESTAS</t>
   </si>
@@ -1031,25 +1031,35 @@
       <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="12" t="s">
-        <v>17</v>
-      </c>
+      <c r="B4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="47">
+        <v>46181</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="I4" s="6"/>
       <c r="J4" t="str">
         <f>IF(F4="✗ No"," ",B4&amp;"-"&amp;C4&amp;"-"&amp;D4&amp;"-"&amp;E4)</f>
-        <v xml:space="preserve"> </v>
+        <v>Francia-Brasil-España-Inglaterra</v>
       </c>
       <c r="K4" t="str" cm="1">
-        <f t="array" ref="K4:K15">_xlfn.UNIQUE(J4:J18)</f>
-        <v xml:space="preserve"> </v>
+        <f t="array" ref="K4:K16">_xlfn.UNIQUE(J4:J18)</f>
+        <v>Francia-Brasil-España-Inglaterra</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1091,16 +1101,16 @@
         <v>45</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>10</v>
-      </c>
       <c r="E6" s="7" t="s">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>14</v>
@@ -1114,10 +1124,10 @@
       <c r="I6" s="6"/>
       <c r="J6" t="str">
         <f t="shared" si="0"/>
-        <v>Francia-España-Argentina-Portugal</v>
+        <v>Portugal-Francia-España-Brasil</v>
       </c>
       <c r="K6" t="str">
-        <v>Francia-España-Argentina-Portugal</v>
+        <v>Portugal-Francia-España-Brasil</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1345,7 +1355,7 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="K13" t="str">
-        <v>Holanda-Inglaterra-Francia-Brasil</v>
+        <v xml:space="preserve"> </v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1362,7 +1372,7 @@
         <v>11</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>14</v>
@@ -1376,10 +1386,10 @@
       <c r="I14" s="6"/>
       <c r="J14" t="str">
         <f t="shared" si="0"/>
-        <v>Holanda-Inglaterra-Francia-Brasil</v>
+        <v>Holanda-Inglaterra-Francia-Alemania</v>
       </c>
       <c r="K14" t="str">
-        <v>España-Brasil-Alemania-Argentina</v>
+        <v>Holanda-Inglaterra-Francia-Alemania</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1403,7 +1413,7 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="K15" t="str">
-        <v>España-Portugal-Francia-Alemania</v>
+        <v>España-Brasil-Alemania-Argentina</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1435,6 +1445,9 @@
       <c r="J16" t="str">
         <f t="shared" si="0"/>
         <v>España-Brasil-Alemania-Argentina</v>
+      </c>
+      <c r="K16" t="str">
+        <v>España-Portugal-Francia-Alemania</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -1982,7 +1995,7 @@
       </c>
       <c r="B2" s="45">
         <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="40"/>
     </row>
@@ -1992,7 +2005,7 @@
       </c>
       <c r="B3" s="42">
         <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")*100000</f>
-        <v>1100000</v>
+        <v>1200000</v>
       </c>
       <c r="C3" s="43"/>
     </row>
@@ -2007,7 +2020,7 @@
       </c>
       <c r="B5" s="42">
         <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")*100000-100000</f>
-        <v>1000000</v>
+        <v>1100000</v>
       </c>
       <c r="C5" s="46" t="s">
         <v>40</v>
@@ -2030,7 +2043,7 @@
       </c>
       <c r="B7" s="42">
         <f>B5+B6</f>
-        <v>1100000</v>
+        <v>1200000</v>
       </c>
       <c r="C7" s="43"/>
     </row>

</xml_diff>

<commit_message>
Se actualiza apuesta de participante
</commit_message>
<xml_diff>
--- a/mundial_2026_apuestas.xlsx
+++ b/mundial_2026_apuestas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1fe95bc314a61fb9/Jupyter/Proyectos/Resultados Mundial 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="131" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0036DAEC-E792-4BFC-9289-A46DAFEAF869}"/>
+  <xr:revisionPtr revIDLastSave="134" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03B030CD-F692-4528-9FC2-8DE2141971F7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="67">
   <si>
     <t>⚽  MUNDIAL 2026 — CONTROL DE APUESTAS</t>
   </si>
@@ -259,6 +259,9 @@
   </si>
   <si>
     <t>Por Definir</t>
+  </si>
+  <si>
+    <t>Japón</t>
   </si>
 </sst>
 </file>
@@ -1206,13 +1209,13 @@
         <v>11</v>
       </c>
       <c r="C9" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>10</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>14</v>
@@ -1226,10 +1229,10 @@
       <c r="I9" s="9"/>
       <c r="J9" t="str">
         <f t="shared" si="0"/>
-        <v>Francia-Inglaterra-España-Argentina</v>
+        <v>Francia-España-Japón-Inglaterra</v>
       </c>
       <c r="K9" t="str">
-        <v>Francia-Inglaterra-España-Argentina</v>
+        <v>Francia-España-Japón-Inglaterra</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Se modifica apuesta e ingresa nuevo participante
</commit_message>
<xml_diff>
--- a/mundial_2026_apuestas.xlsx
+++ b/mundial_2026_apuestas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1fe95bc314a61fb9/Jupyter/Proyectos/Resultados Mundial 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="134" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03B030CD-F692-4528-9FC2-8DE2141971F7}"/>
+  <xr:revisionPtr revIDLastSave="146" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8848AF78-1D76-4C82-8E9E-578301768ADD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="67">
   <si>
     <t>⚽  MUNDIAL 2026 — CONTROL DE APUESTAS</t>
   </si>
@@ -1061,7 +1061,7 @@
         <v>Francia-Brasil-España-Inglaterra</v>
       </c>
       <c r="K4" t="str" cm="1">
-        <f t="array" ref="K4:K16">_xlfn.UNIQUE(J4:J18)</f>
+        <f t="array" ref="K4:K17">_xlfn.UNIQUE(J4:J18)</f>
         <v>Francia-Brasil-España-Inglaterra</v>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="K15" t="str">
-        <v>España-Brasil-Alemania-Argentina</v>
+        <v>Brasil-España-Francia-Portugal</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1424,16 +1424,16 @@
         <v>55</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>12</v>
-      </c>
       <c r="D16" s="7" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>14</v>
@@ -1447,13 +1447,13 @@
       <c r="I16" s="6"/>
       <c r="J16" t="str">
         <f t="shared" si="0"/>
-        <v>España-Brasil-Alemania-Argentina</v>
+        <v>Brasil-España-Francia-Portugal</v>
       </c>
       <c r="K16" t="str">
         <v>España-Portugal-Francia-Alemania</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>56</v>
       </c>
@@ -1483,26 +1483,39 @@
         <f t="shared" si="0"/>
         <v>España-Portugal-Francia-Alemania</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K17" t="str">
+        <v>Francia-Brasil-España-Alemania</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="G18" s="47"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="12" t="s">
-        <v>17</v>
-      </c>
+      <c r="B18" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="47">
+        <v>46183</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="I18" s="6"/>
       <c r="J18" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
+        <v>Francia-Brasil-España-Alemania</v>
       </c>
     </row>
   </sheetData>
@@ -1998,7 +2011,7 @@
       </c>
       <c r="B2" s="45">
         <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="40"/>
     </row>
@@ -2008,7 +2021,7 @@
       </c>
       <c r="B3" s="42">
         <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")*100000</f>
-        <v>1200000</v>
+        <v>1300000</v>
       </c>
       <c r="C3" s="43"/>
     </row>
@@ -2023,7 +2036,7 @@
       </c>
       <c r="B5" s="42">
         <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")*100000-100000</f>
-        <v>1100000</v>
+        <v>1200000</v>
       </c>
       <c r="C5" s="46" t="s">
         <v>40</v>
@@ -2046,7 +2059,7 @@
       </c>
       <c r="B7" s="42">
         <f>B5+B6</f>
-        <v>1200000</v>
+        <v>1300000</v>
       </c>
       <c r="C7" s="43"/>
     </row>

</xml_diff>

<commit_message>
Entra nuevo participante y se actualiza premio al 2do lugar.
</commit_message>
<xml_diff>
--- a/mundial_2026_apuestas.xlsx
+++ b/mundial_2026_apuestas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1fe95bc314a61fb9/Jupyter/Proyectos/Resultados Mundial 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="146" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8848AF78-1D76-4C82-8E9E-578301768ADD}"/>
+  <xr:revisionPtr revIDLastSave="162" documentId="11_71424545E5A34E169FA4A7C6E2A60B7FBE6F0FF7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7BBA099-56A9-4B21-A95D-E9020852DD20}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="67">
   <si>
     <t>⚽  MUNDIAL 2026 — CONTROL DE APUESTAS</t>
   </si>
@@ -90,9 +90,6 @@
     <t>Observaciones</t>
   </si>
   <si>
-    <t>Carlos</t>
-  </si>
-  <si>
     <t>Argentina</t>
   </si>
   <si>
@@ -183,15 +180,9 @@
     <t>Premio 1° lugar ($)</t>
   </si>
   <si>
-    <t>Pozo total − $100.000</t>
-  </si>
-  <si>
     <t>Premio 2° lugar ($)</t>
   </si>
   <si>
-    <t>$100.000 fijo</t>
-  </si>
-  <si>
     <t>Total premios ($)</t>
   </si>
   <si>
@@ -219,9 +210,6 @@
     <t>Juan Reveco</t>
   </si>
   <si>
-    <t>Kote</t>
-  </si>
-  <si>
     <t>Manuel</t>
   </si>
   <si>
@@ -262,6 +250,18 @@
   </si>
   <si>
     <t>Japón</t>
+  </si>
+  <si>
+    <t>Carlos Aliaga</t>
+  </si>
+  <si>
+    <t>Carlos Navarro</t>
+  </si>
+  <si>
+    <t>$200.000 fijo</t>
+  </si>
+  <si>
+    <t>Pozo total − $200.000</t>
   </si>
 </sst>
 </file>
@@ -1017,10 +1017,10 @@
         <v>7</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>8</v>
@@ -1032,28 +1032,28 @@
     </row>
     <row r="4" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>9</v>
+        <v>63</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G4" s="47">
         <v>46181</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I4" s="6"/>
       <c r="J4" t="str">
@@ -1061,34 +1061,34 @@
         <v>Francia-Brasil-España-Inglaterra</v>
       </c>
       <c r="K4" t="str" cm="1">
-        <f t="array" ref="K4:K17">_xlfn.UNIQUE(J4:J18)</f>
+        <f t="array" ref="K4:K18">_xlfn.UNIQUE(J4:J18)</f>
         <v>Francia-Brasil-España-Inglaterra</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G5" s="48">
         <v>46175</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I5" s="9"/>
       <c r="J5" t="str">
@@ -1101,28 +1101,28 @@
     </row>
     <row r="6" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G6" s="47">
         <v>46174</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I6" s="6"/>
       <c r="J6" t="str">
@@ -1135,28 +1135,28 @@
     </row>
     <row r="7" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G7" s="48">
         <v>46174</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I7" s="9"/>
       <c r="J7" t="str">
@@ -1169,28 +1169,28 @@
     </row>
     <row r="8" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G8" s="47">
         <v>46176</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I8" s="6"/>
       <c r="J8" t="str">
@@ -1203,28 +1203,28 @@
     </row>
     <row r="9" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G9" s="48">
         <v>46175</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" t="str">
@@ -1237,28 +1237,28 @@
     </row>
     <row r="10" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E10" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G10" s="47">
         <v>46178</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I10" s="6"/>
       <c r="J10" t="str">
@@ -1271,28 +1271,28 @@
     </row>
     <row r="11" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G11" s="48">
         <v>46174</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I11" s="9"/>
       <c r="J11" t="str">
@@ -1305,28 +1305,28 @@
     </row>
     <row r="12" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B12" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G12" s="47">
         <v>46176</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I12" s="6"/>
       <c r="J12" t="str">
@@ -1339,52 +1339,62 @@
     </row>
     <row r="13" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" s="48"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="12" t="s">
-        <v>17</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="48">
+        <v>46184</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="I13" s="9"/>
       <c r="J13" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
+        <v>Argentina-Portugal-España-Francia</v>
       </c>
       <c r="K13" t="str">
-        <v xml:space="preserve"> </v>
+        <v>Argentina-Portugal-España-Francia</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G14" s="47">
         <v>46175</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I14" s="6"/>
       <c r="J14" t="str">
@@ -1397,52 +1407,52 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G15" s="48"/>
       <c r="H15" s="10"/>
       <c r="I15" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J15" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="K15" t="str">
-        <v>Brasil-España-Francia-Portugal</v>
+        <v xml:space="preserve"> </v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="7" t="s">
+      <c r="F16" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G16" s="47">
         <v>46176</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I16" s="6"/>
       <c r="J16" t="str">
@@ -1450,33 +1460,33 @@
         <v>Brasil-España-Francia-Portugal</v>
       </c>
       <c r="K16" t="str">
-        <v>España-Portugal-Francia-Alemania</v>
+        <v>Brasil-España-Francia-Portugal</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B17" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G17" s="48">
         <v>46178</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I17" s="9"/>
       <c r="J17" t="str">
@@ -1484,37 +1494,40 @@
         <v>España-Portugal-Francia-Alemania</v>
       </c>
       <c r="K17" t="str">
-        <v>Francia-Brasil-España-Alemania</v>
+        <v>España-Portugal-Francia-Alemania</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="E18" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G18" s="47">
         <v>46183</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I18" s="6"/>
       <c r="J18" t="str">
         <f t="shared" si="0"/>
+        <v>Francia-Brasil-España-Alemania</v>
+      </c>
+      <c r="K18" t="str">
         <v>Francia-Brasil-España-Alemania</v>
       </c>
     </row>
@@ -1540,35 +1553,35 @@
   <sheetData>
     <row r="1" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="51" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B1" s="51"/>
       <c r="C1" s="51"/>
     </row>
     <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="52" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B2" s="52"/>
       <c r="C2" s="52"/>
     </row>
     <row r="3" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="C3" s="13" t="s">
         <v>21</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C4" s="16">
         <v>4</v>
@@ -1576,10 +1589,10 @@
     </row>
     <row r="5" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C5" s="16">
         <v>3</v>
@@ -1587,10 +1600,10 @@
     </row>
     <row r="6" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C6" s="16">
         <v>2</v>
@@ -1598,10 +1611,10 @@
     </row>
     <row r="7" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C7" s="16">
         <v>1</v>
@@ -1630,7 +1643,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="51" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B1" s="51"/>
       <c r="C1" s="51"/>
@@ -1642,7 +1655,7 @@
     </row>
     <row r="2" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="52" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B2" s="52"/>
       <c r="C2" s="52"/>
@@ -1654,28 +1667,28 @@
     </row>
     <row r="3" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1684,7 +1697,7 @@
       </c>
       <c r="B4" s="21" t="str">
         <f>Apuestas!A4</f>
-        <v>Carlos</v>
+        <v>Carlos Aliaga</v>
       </c>
       <c r="C4" s="22">
         <f>IF(Apuestas!B4='Resultados Oficiales'!$B$4,4,0)</f>
@@ -1954,7 +1967,7 @@
       </c>
       <c r="B13" s="33" t="str">
         <f>Apuestas!A13</f>
-        <v>Kote</v>
+        <v>Carlos Navarro</v>
       </c>
       <c r="C13" s="7">
         <f>IF(Apuestas!B13='Resultados Oficiales'!$B$4,4,0)</f>
@@ -2000,28 +2013,28 @@
   <sheetData>
     <row r="1" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="51" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B1" s="51"/>
       <c r="C1" s="51"/>
     </row>
     <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="45">
         <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" s="40"/>
     </row>
     <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="42">
         <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")*100000</f>
-        <v>1300000</v>
+        <v>1400000</v>
       </c>
       <c r="C3" s="43"/>
     </row>
@@ -2032,34 +2045,34 @@
     </row>
     <row r="5" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="42">
-        <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")*100000-100000</f>
+        <f>COUNTIF(Apuestas!F4:F18,"✓ Sí")*100000-200000</f>
         <v>1200000</v>
       </c>
       <c r="C5" s="46" t="s">
-        <v>40</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="38" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B6" s="39">
-        <v>100000</v>
+        <v>200000</v>
       </c>
       <c r="C6" s="46" t="s">
-        <v>42</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B7" s="42">
         <f>B5+B6</f>
-        <v>1300000</v>
+        <v>1400000</v>
       </c>
       <c r="C7" s="43"/>
     </row>

</xml_diff>